<commit_message>
feat: white-themed mobile-first dashboard with A4 print and Gujarati tracking columns
</commit_message>
<xml_diff>
--- a/Maitry_and_Smit_Invitation_List_18_Oct.xlsx
+++ b/Maitry_and_Smit_Invitation_List_18_Oct.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -540,10 +540,12 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -556,7 +558,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Contacts: 94  |  Sent: 51  |  Pending: 43  |  Updated: 18-Oct-2026 09:50 PM</t>
+          <t>Total Contacts: 94  |  Sent: 51  |  Pending: 43  |  Updated: 18-Oct-2026 10:07 PM</t>
         </is>
       </c>
     </row>
@@ -612,6 +614,16 @@
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>વોટ્સએપ OK</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>ફોન પર વાતચીત</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -662,7 +674,9 @@
           <t>2026-10-18 21:21:22</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
+      <c r="L4" s="4" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -709,7 +723,9 @@
           <t>2026-10-18 21:21:40</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -756,7 +772,9 @@
           <t>2026-10-18 21:21:59</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -803,7 +821,9 @@
           <t>2026-10-18 21:22:21</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -850,7 +870,9 @@
           <t>2026-10-18 21:22:43</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -897,7 +919,9 @@
           <t>2026-10-18 21:23:08</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -944,7 +968,9 @@
           <t>2026-10-18 21:23:31</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="n">
@@ -995,7 +1021,9 @@
           <t>2026-10-18 21:23:50</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -1042,7 +1070,9 @@
           <t>2026-10-18 21:24:09</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -1089,7 +1119,9 @@
           <t>2026-10-18 21:24:33</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -1136,7 +1168,9 @@
           <t>2026-10-18 21:24:52</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -1183,7 +1217,9 @@
           <t>2026-10-18 21:25:11</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="n">
@@ -1230,7 +1266,9 @@
           <t>2026-10-18 21:25:31</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -1277,7 +1315,9 @@
           <t>2026-10-18 21:25:55</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -1324,7 +1364,9 @@
           <t>2026-10-18 21:26:16</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -1371,7 +1413,9 @@
           <t>2026-10-18 21:26:35</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -1418,7 +1462,9 @@
           <t>2026-10-18 21:26:55</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="4" t="n">
@@ -1465,7 +1511,9 @@
           <t>2026-10-18 21:27:15</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr"/>
+      <c r="M21" s="5" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="4" t="n">
@@ -1512,7 +1560,9 @@
           <t>2026-10-18 21:27:37</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -1563,7 +1613,9 @@
           <t>2026-10-18 21:27:56</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="5" t="inlineStr"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="4" t="n">
@@ -1610,7 +1662,9 @@
           <t>2026-10-18 21:28:14</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -1657,7 +1711,9 @@
           <t>2026-10-18 21:28:34</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1704,7 +1760,9 @@
           <t>2026-10-18 21:28:52</t>
         </is>
       </c>
-      <c r="K26" s="5" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -1751,7 +1809,9 @@
           <t>2026-10-18 21:29:17</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr"/>
+      <c r="M27" s="5" t="inlineStr"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="4" t="n">
@@ -1798,7 +1858,9 @@
           <t>2026-10-18 21:29:36</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="5" t="inlineStr"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="4" t="n">
@@ -1845,7 +1907,9 @@
           <t>2026-10-18 21:30:25</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
+      <c r="L29" s="4" t="inlineStr"/>
+      <c r="M29" s="5" t="inlineStr"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1892,7 +1956,9 @@
           <t>2026-10-18 21:30:46</t>
         </is>
       </c>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
+      <c r="L30" s="4" t="inlineStr"/>
+      <c r="M30" s="5" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="4" t="n">
@@ -1939,7 +2005,9 @@
           <t>2026-10-18 21:31:09</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr"/>
+      <c r="M31" s="5" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="4" t="n">
@@ -1986,7 +2054,9 @@
           <t>2026-10-18 21:31:36</t>
         </is>
       </c>
-      <c r="K32" s="5" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr"/>
+      <c r="M32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="4" t="n">
@@ -2033,7 +2103,9 @@
           <t>2026-10-18 21:31:58</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr"/>
+      <c r="M33" s="5" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="8" t="n">
@@ -2068,7 +2140,9 @@
       <c r="H34" s="10" t="inlineStr"/>
       <c r="I34" s="9" t="inlineStr"/>
       <c r="J34" s="8" t="inlineStr"/>
-      <c r="K34" s="9" t="inlineStr"/>
+      <c r="K34" s="8" t="inlineStr"/>
+      <c r="L34" s="8" t="inlineStr"/>
+      <c r="M34" s="9" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="11" t="n">
@@ -2103,7 +2177,9 @@
       <c r="H35" s="13" t="inlineStr"/>
       <c r="I35" s="12" t="inlineStr"/>
       <c r="J35" s="11" t="inlineStr"/>
-      <c r="K35" s="12" t="inlineStr"/>
+      <c r="K35" s="11" t="inlineStr"/>
+      <c r="L35" s="11" t="inlineStr"/>
+      <c r="M35" s="12" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="8" t="n">
@@ -2138,7 +2214,9 @@
       <c r="H36" s="10" t="inlineStr"/>
       <c r="I36" s="9" t="inlineStr"/>
       <c r="J36" s="8" t="inlineStr"/>
-      <c r="K36" s="9" t="inlineStr"/>
+      <c r="K36" s="8" t="inlineStr"/>
+      <c r="L36" s="8" t="inlineStr"/>
+      <c r="M36" s="9" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="11" t="n">
@@ -2173,7 +2251,9 @@
       <c r="H37" s="13" t="inlineStr"/>
       <c r="I37" s="12" t="inlineStr"/>
       <c r="J37" s="11" t="inlineStr"/>
-      <c r="K37" s="12" t="inlineStr"/>
+      <c r="K37" s="11" t="inlineStr"/>
+      <c r="L37" s="11" t="inlineStr"/>
+      <c r="M37" s="12" t="inlineStr"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="8" t="n">
@@ -2208,7 +2288,9 @@
       <c r="H38" s="10" t="inlineStr"/>
       <c r="I38" s="9" t="inlineStr"/>
       <c r="J38" s="8" t="inlineStr"/>
-      <c r="K38" s="9" t="inlineStr"/>
+      <c r="K38" s="8" t="inlineStr"/>
+      <c r="L38" s="8" t="inlineStr"/>
+      <c r="M38" s="9" t="inlineStr"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="11" t="n">
@@ -2247,7 +2329,9 @@
       <c r="H39" s="13" t="inlineStr"/>
       <c r="I39" s="12" t="inlineStr"/>
       <c r="J39" s="11" t="inlineStr"/>
-      <c r="K39" s="12" t="inlineStr"/>
+      <c r="K39" s="11" t="inlineStr"/>
+      <c r="L39" s="11" t="inlineStr"/>
+      <c r="M39" s="12" t="inlineStr"/>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="8" t="n">
@@ -2282,7 +2366,9 @@
       <c r="H40" s="10" t="inlineStr"/>
       <c r="I40" s="9" t="inlineStr"/>
       <c r="J40" s="8" t="inlineStr"/>
-      <c r="K40" s="9" t="inlineStr"/>
+      <c r="K40" s="8" t="inlineStr"/>
+      <c r="L40" s="8" t="inlineStr"/>
+      <c r="M40" s="9" t="inlineStr"/>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="11" t="n">
@@ -2317,7 +2403,9 @@
       <c r="H41" s="13" t="inlineStr"/>
       <c r="I41" s="12" t="inlineStr"/>
       <c r="J41" s="11" t="inlineStr"/>
-      <c r="K41" s="12" t="inlineStr"/>
+      <c r="K41" s="11" t="inlineStr"/>
+      <c r="L41" s="11" t="inlineStr"/>
+      <c r="M41" s="12" t="inlineStr"/>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="8" t="n">
@@ -2352,7 +2440,9 @@
       <c r="H42" s="10" t="inlineStr"/>
       <c r="I42" s="9" t="inlineStr"/>
       <c r="J42" s="8" t="inlineStr"/>
-      <c r="K42" s="9" t="inlineStr"/>
+      <c r="K42" s="8" t="inlineStr"/>
+      <c r="L42" s="8" t="inlineStr"/>
+      <c r="M42" s="9" t="inlineStr"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="11" t="n">
@@ -2387,7 +2477,9 @@
       <c r="H43" s="13" t="inlineStr"/>
       <c r="I43" s="12" t="inlineStr"/>
       <c r="J43" s="11" t="inlineStr"/>
-      <c r="K43" s="12" t="inlineStr"/>
+      <c r="K43" s="11" t="inlineStr"/>
+      <c r="L43" s="11" t="inlineStr"/>
+      <c r="M43" s="12" t="inlineStr"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="8" t="n">
@@ -2422,7 +2514,9 @@
       <c r="H44" s="10" t="inlineStr"/>
       <c r="I44" s="9" t="inlineStr"/>
       <c r="J44" s="8" t="inlineStr"/>
-      <c r="K44" s="9" t="inlineStr"/>
+      <c r="K44" s="8" t="inlineStr"/>
+      <c r="L44" s="8" t="inlineStr"/>
+      <c r="M44" s="9" t="inlineStr"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="11" t="n">
@@ -2461,7 +2555,9 @@
       <c r="H45" s="13" t="inlineStr"/>
       <c r="I45" s="12" t="inlineStr"/>
       <c r="J45" s="11" t="inlineStr"/>
-      <c r="K45" s="12" t="inlineStr"/>
+      <c r="K45" s="11" t="inlineStr"/>
+      <c r="L45" s="11" t="inlineStr"/>
+      <c r="M45" s="12" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="8" t="n">
@@ -2500,7 +2596,9 @@
       <c r="H46" s="10" t="inlineStr"/>
       <c r="I46" s="9" t="inlineStr"/>
       <c r="J46" s="8" t="inlineStr"/>
-      <c r="K46" s="9" t="inlineStr"/>
+      <c r="K46" s="8" t="inlineStr"/>
+      <c r="L46" s="8" t="inlineStr"/>
+      <c r="M46" s="9" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="11" t="n">
@@ -2535,7 +2633,9 @@
       <c r="H47" s="13" t="inlineStr"/>
       <c r="I47" s="12" t="inlineStr"/>
       <c r="J47" s="11" t="inlineStr"/>
-      <c r="K47" s="12" t="inlineStr"/>
+      <c r="K47" s="11" t="inlineStr"/>
+      <c r="L47" s="11" t="inlineStr"/>
+      <c r="M47" s="12" t="inlineStr"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="8" t="n">
@@ -2574,7 +2674,9 @@
       <c r="H48" s="10" t="inlineStr"/>
       <c r="I48" s="9" t="inlineStr"/>
       <c r="J48" s="8" t="inlineStr"/>
-      <c r="K48" s="9" t="inlineStr"/>
+      <c r="K48" s="8" t="inlineStr"/>
+      <c r="L48" s="8" t="inlineStr"/>
+      <c r="M48" s="9" t="inlineStr"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="11" t="n">
@@ -2609,7 +2711,9 @@
       <c r="H49" s="13" t="inlineStr"/>
       <c r="I49" s="12" t="inlineStr"/>
       <c r="J49" s="11" t="inlineStr"/>
-      <c r="K49" s="12" t="inlineStr"/>
+      <c r="K49" s="11" t="inlineStr"/>
+      <c r="L49" s="11" t="inlineStr"/>
+      <c r="M49" s="12" t="inlineStr"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="8" t="n">
@@ -2644,7 +2748,9 @@
       <c r="H50" s="10" t="inlineStr"/>
       <c r="I50" s="9" t="inlineStr"/>
       <c r="J50" s="8" t="inlineStr"/>
-      <c r="K50" s="9" t="inlineStr"/>
+      <c r="K50" s="8" t="inlineStr"/>
+      <c r="L50" s="8" t="inlineStr"/>
+      <c r="M50" s="9" t="inlineStr"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="11" t="n">
@@ -2679,7 +2785,9 @@
       <c r="H51" s="13" t="inlineStr"/>
       <c r="I51" s="12" t="inlineStr"/>
       <c r="J51" s="11" t="inlineStr"/>
-      <c r="K51" s="12" t="inlineStr"/>
+      <c r="K51" s="11" t="inlineStr"/>
+      <c r="L51" s="11" t="inlineStr"/>
+      <c r="M51" s="12" t="inlineStr"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="8" t="n">
@@ -2714,7 +2822,9 @@
       <c r="H52" s="10" t="inlineStr"/>
       <c r="I52" s="9" t="inlineStr"/>
       <c r="J52" s="8" t="inlineStr"/>
-      <c r="K52" s="9" t="inlineStr"/>
+      <c r="K52" s="8" t="inlineStr"/>
+      <c r="L52" s="8" t="inlineStr"/>
+      <c r="M52" s="9" t="inlineStr"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="11" t="n">
@@ -2753,7 +2863,9 @@
       <c r="H53" s="13" t="inlineStr"/>
       <c r="I53" s="12" t="inlineStr"/>
       <c r="J53" s="11" t="inlineStr"/>
-      <c r="K53" s="12" t="inlineStr"/>
+      <c r="K53" s="11" t="inlineStr"/>
+      <c r="L53" s="11" t="inlineStr"/>
+      <c r="M53" s="12" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="8" t="n">
@@ -2788,7 +2900,9 @@
       <c r="H54" s="10" t="inlineStr"/>
       <c r="I54" s="9" t="inlineStr"/>
       <c r="J54" s="8" t="inlineStr"/>
-      <c r="K54" s="9" t="inlineStr"/>
+      <c r="K54" s="8" t="inlineStr"/>
+      <c r="L54" s="8" t="inlineStr"/>
+      <c r="M54" s="9" t="inlineStr"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="11" t="n">
@@ -2823,7 +2937,9 @@
       <c r="H55" s="13" t="inlineStr"/>
       <c r="I55" s="12" t="inlineStr"/>
       <c r="J55" s="11" t="inlineStr"/>
-      <c r="K55" s="12" t="inlineStr"/>
+      <c r="K55" s="11" t="inlineStr"/>
+      <c r="L55" s="11" t="inlineStr"/>
+      <c r="M55" s="12" t="inlineStr"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="8" t="n">
@@ -2858,7 +2974,9 @@
       <c r="H56" s="10" t="inlineStr"/>
       <c r="I56" s="9" t="inlineStr"/>
       <c r="J56" s="8" t="inlineStr"/>
-      <c r="K56" s="9" t="inlineStr"/>
+      <c r="K56" s="8" t="inlineStr"/>
+      <c r="L56" s="8" t="inlineStr"/>
+      <c r="M56" s="9" t="inlineStr"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="11" t="n">
@@ -2893,7 +3011,9 @@
       <c r="H57" s="13" t="inlineStr"/>
       <c r="I57" s="12" t="inlineStr"/>
       <c r="J57" s="11" t="inlineStr"/>
-      <c r="K57" s="12" t="inlineStr"/>
+      <c r="K57" s="11" t="inlineStr"/>
+      <c r="L57" s="11" t="inlineStr"/>
+      <c r="M57" s="12" t="inlineStr"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="8" t="n">
@@ -2928,7 +3048,9 @@
       <c r="H58" s="10" t="inlineStr"/>
       <c r="I58" s="9" t="inlineStr"/>
       <c r="J58" s="8" t="inlineStr"/>
-      <c r="K58" s="9" t="inlineStr"/>
+      <c r="K58" s="8" t="inlineStr"/>
+      <c r="L58" s="8" t="inlineStr"/>
+      <c r="M58" s="9" t="inlineStr"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="11" t="n">
@@ -2963,7 +3085,9 @@
       <c r="H59" s="13" t="inlineStr"/>
       <c r="I59" s="12" t="inlineStr"/>
       <c r="J59" s="11" t="inlineStr"/>
-      <c r="K59" s="12" t="inlineStr"/>
+      <c r="K59" s="11" t="inlineStr"/>
+      <c r="L59" s="11" t="inlineStr"/>
+      <c r="M59" s="12" t="inlineStr"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="8" t="n">
@@ -2998,7 +3122,9 @@
       <c r="H60" s="10" t="inlineStr"/>
       <c r="I60" s="9" t="inlineStr"/>
       <c r="J60" s="8" t="inlineStr"/>
-      <c r="K60" s="9" t="inlineStr"/>
+      <c r="K60" s="8" t="inlineStr"/>
+      <c r="L60" s="8" t="inlineStr"/>
+      <c r="M60" s="9" t="inlineStr"/>
     </row>
     <row r="61" ht="20" customHeight="1">
       <c r="A61" s="11" t="n">
@@ -3033,7 +3159,9 @@
       <c r="H61" s="13" t="inlineStr"/>
       <c r="I61" s="12" t="inlineStr"/>
       <c r="J61" s="11" t="inlineStr"/>
-      <c r="K61" s="12" t="inlineStr"/>
+      <c r="K61" s="11" t="inlineStr"/>
+      <c r="L61" s="11" t="inlineStr"/>
+      <c r="M61" s="12" t="inlineStr"/>
     </row>
     <row r="62" ht="20" customHeight="1">
       <c r="A62" s="8" t="n">
@@ -3068,7 +3196,9 @@
       <c r="H62" s="10" t="inlineStr"/>
       <c r="I62" s="9" t="inlineStr"/>
       <c r="J62" s="8" t="inlineStr"/>
-      <c r="K62" s="9" t="inlineStr"/>
+      <c r="K62" s="8" t="inlineStr"/>
+      <c r="L62" s="8" t="inlineStr"/>
+      <c r="M62" s="9" t="inlineStr"/>
     </row>
     <row r="63" ht="20" customHeight="1">
       <c r="A63" s="11" t="n">
@@ -3103,7 +3233,9 @@
       <c r="H63" s="13" t="inlineStr"/>
       <c r="I63" s="12" t="inlineStr"/>
       <c r="J63" s="11" t="inlineStr"/>
-      <c r="K63" s="12" t="inlineStr"/>
+      <c r="K63" s="11" t="inlineStr"/>
+      <c r="L63" s="11" t="inlineStr"/>
+      <c r="M63" s="12" t="inlineStr"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="8" t="n">
@@ -3138,7 +3270,9 @@
       <c r="H64" s="10" t="inlineStr"/>
       <c r="I64" s="9" t="inlineStr"/>
       <c r="J64" s="8" t="inlineStr"/>
-      <c r="K64" s="9" t="inlineStr"/>
+      <c r="K64" s="8" t="inlineStr"/>
+      <c r="L64" s="8" t="inlineStr"/>
+      <c r="M64" s="9" t="inlineStr"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="A65" s="11" t="n">
@@ -3173,7 +3307,9 @@
       <c r="H65" s="13" t="inlineStr"/>
       <c r="I65" s="12" t="inlineStr"/>
       <c r="J65" s="11" t="inlineStr"/>
-      <c r="K65" s="12" t="inlineStr"/>
+      <c r="K65" s="11" t="inlineStr"/>
+      <c r="L65" s="11" t="inlineStr"/>
+      <c r="M65" s="12" t="inlineStr"/>
     </row>
     <row r="66" ht="20" customHeight="1">
       <c r="A66" s="8" t="n">
@@ -3208,7 +3344,9 @@
       <c r="H66" s="10" t="inlineStr"/>
       <c r="I66" s="9" t="inlineStr"/>
       <c r="J66" s="8" t="inlineStr"/>
-      <c r="K66" s="9" t="inlineStr"/>
+      <c r="K66" s="8" t="inlineStr"/>
+      <c r="L66" s="8" t="inlineStr"/>
+      <c r="M66" s="9" t="inlineStr"/>
     </row>
     <row r="67" ht="20" customHeight="1">
       <c r="A67" s="11" t="n">
@@ -3243,7 +3381,9 @@
       <c r="H67" s="13" t="inlineStr"/>
       <c r="I67" s="12" t="inlineStr"/>
       <c r="J67" s="11" t="inlineStr"/>
-      <c r="K67" s="12" t="inlineStr"/>
+      <c r="K67" s="11" t="inlineStr"/>
+      <c r="L67" s="11" t="inlineStr"/>
+      <c r="M67" s="12" t="inlineStr"/>
     </row>
     <row r="68" ht="20" customHeight="1">
       <c r="A68" s="8" t="n">
@@ -3278,7 +3418,9 @@
       <c r="H68" s="10" t="inlineStr"/>
       <c r="I68" s="9" t="inlineStr"/>
       <c r="J68" s="8" t="inlineStr"/>
-      <c r="K68" s="9" t="inlineStr"/>
+      <c r="K68" s="8" t="inlineStr"/>
+      <c r="L68" s="8" t="inlineStr"/>
+      <c r="M68" s="9" t="inlineStr"/>
     </row>
     <row r="69" ht="20" customHeight="1">
       <c r="A69" s="11" t="n">
@@ -3313,7 +3455,9 @@
       <c r="H69" s="13" t="inlineStr"/>
       <c r="I69" s="12" t="inlineStr"/>
       <c r="J69" s="11" t="inlineStr"/>
-      <c r="K69" s="12" t="inlineStr"/>
+      <c r="K69" s="11" t="inlineStr"/>
+      <c r="L69" s="11" t="inlineStr"/>
+      <c r="M69" s="12" t="inlineStr"/>
     </row>
     <row r="70" ht="20" customHeight="1">
       <c r="A70" s="8" t="n">
@@ -3348,7 +3492,9 @@
       <c r="H70" s="10" t="inlineStr"/>
       <c r="I70" s="9" t="inlineStr"/>
       <c r="J70" s="8" t="inlineStr"/>
-      <c r="K70" s="9" t="inlineStr"/>
+      <c r="K70" s="8" t="inlineStr"/>
+      <c r="L70" s="8" t="inlineStr"/>
+      <c r="M70" s="9" t="inlineStr"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="11" t="n">
@@ -3383,7 +3529,9 @@
       <c r="H71" s="13" t="inlineStr"/>
       <c r="I71" s="12" t="inlineStr"/>
       <c r="J71" s="11" t="inlineStr"/>
-      <c r="K71" s="12" t="inlineStr"/>
+      <c r="K71" s="11" t="inlineStr"/>
+      <c r="L71" s="11" t="inlineStr"/>
+      <c r="M71" s="12" t="inlineStr"/>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="8" t="n">
@@ -3418,7 +3566,9 @@
       <c r="H72" s="10" t="inlineStr"/>
       <c r="I72" s="9" t="inlineStr"/>
       <c r="J72" s="8" t="inlineStr"/>
-      <c r="K72" s="9" t="inlineStr"/>
+      <c r="K72" s="8" t="inlineStr"/>
+      <c r="L72" s="8" t="inlineStr"/>
+      <c r="M72" s="9" t="inlineStr"/>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="11" t="n">
@@ -3453,7 +3603,9 @@
       <c r="H73" s="13" t="inlineStr"/>
       <c r="I73" s="12" t="inlineStr"/>
       <c r="J73" s="11" t="inlineStr"/>
-      <c r="K73" s="12" t="inlineStr"/>
+      <c r="K73" s="11" t="inlineStr"/>
+      <c r="L73" s="11" t="inlineStr"/>
+      <c r="M73" s="12" t="inlineStr"/>
     </row>
     <row r="74" ht="20" customHeight="1">
       <c r="A74" s="8" t="n">
@@ -3488,7 +3640,9 @@
       <c r="H74" s="10" t="inlineStr"/>
       <c r="I74" s="9" t="inlineStr"/>
       <c r="J74" s="8" t="inlineStr"/>
-      <c r="K74" s="9" t="inlineStr"/>
+      <c r="K74" s="8" t="inlineStr"/>
+      <c r="L74" s="8" t="inlineStr"/>
+      <c r="M74" s="9" t="inlineStr"/>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="11" t="n">
@@ -3523,7 +3677,9 @@
       <c r="H75" s="13" t="inlineStr"/>
       <c r="I75" s="12" t="inlineStr"/>
       <c r="J75" s="11" t="inlineStr"/>
-      <c r="K75" s="12" t="inlineStr"/>
+      <c r="K75" s="11" t="inlineStr"/>
+      <c r="L75" s="11" t="inlineStr"/>
+      <c r="M75" s="12" t="inlineStr"/>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="8" t="n">
@@ -3558,7 +3714,9 @@
       <c r="H76" s="10" t="inlineStr"/>
       <c r="I76" s="9" t="inlineStr"/>
       <c r="J76" s="8" t="inlineStr"/>
-      <c r="K76" s="9" t="inlineStr"/>
+      <c r="K76" s="8" t="inlineStr"/>
+      <c r="L76" s="8" t="inlineStr"/>
+      <c r="M76" s="9" t="inlineStr"/>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="4" t="n">
@@ -3605,7 +3763,9 @@
           <t>2026-10-18 21:39:55</t>
         </is>
       </c>
-      <c r="K77" s="5" t="inlineStr"/>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+      <c r="M77" s="5" t="inlineStr"/>
     </row>
     <row r="78" ht="20" customHeight="1">
       <c r="A78" s="4" t="n">
@@ -3652,7 +3812,9 @@
           <t>2026-10-18 21:40:15</t>
         </is>
       </c>
-      <c r="K78" s="5" t="inlineStr"/>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
     </row>
     <row r="79" ht="20" customHeight="1">
       <c r="A79" s="4" t="n">
@@ -3699,7 +3861,9 @@
           <t>2026-10-18 21:40:34</t>
         </is>
       </c>
-      <c r="K79" s="5" t="inlineStr"/>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
     </row>
     <row r="80" ht="20" customHeight="1">
       <c r="A80" s="4" t="n">
@@ -3746,7 +3910,9 @@
           <t>2026-10-18 21:40:52</t>
         </is>
       </c>
-      <c r="K80" s="5" t="inlineStr"/>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
     </row>
     <row r="81" ht="20" customHeight="1">
       <c r="A81" s="4" t="n">
@@ -3793,7 +3959,9 @@
           <t>2026-10-18 21:41:11</t>
         </is>
       </c>
-      <c r="K81" s="5" t="inlineStr"/>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+      <c r="M81" s="5" t="inlineStr"/>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="4" t="n">
@@ -3840,7 +4008,9 @@
           <t>2026-10-18 21:41:34</t>
         </is>
       </c>
-      <c r="K82" s="5" t="inlineStr"/>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+      <c r="M82" s="5" t="inlineStr"/>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="4" t="n">
@@ -3887,7 +4057,9 @@
           <t>2026-10-18 21:50:08</t>
         </is>
       </c>
-      <c r="K83" s="5" t="inlineStr"/>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+      <c r="M83" s="5" t="inlineStr"/>
     </row>
     <row r="84" ht="20" customHeight="1">
       <c r="A84" s="4" t="n">
@@ -3934,7 +4106,9 @@
           <t>2026-10-18 21:42:11</t>
         </is>
       </c>
-      <c r="K84" s="5" t="inlineStr"/>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+      <c r="M84" s="5" t="inlineStr"/>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="4" t="n">
@@ -3981,7 +4155,9 @@
           <t>2026-10-18 21:42:31</t>
         </is>
       </c>
-      <c r="K85" s="5" t="inlineStr"/>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="5" t="inlineStr"/>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="4" t="n">
@@ -4028,7 +4204,9 @@
           <t>2026-10-18 21:42:49</t>
         </is>
       </c>
-      <c r="K86" s="5" t="inlineStr"/>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+      <c r="M86" s="5" t="inlineStr"/>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="4" t="n">
@@ -4075,7 +4253,9 @@
           <t>2026-10-18 21:50:08</t>
         </is>
       </c>
-      <c r="K87" s="5" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="5" t="inlineStr"/>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="4" t="n">
@@ -4122,7 +4302,9 @@
           <t>2026-10-18 21:43:24</t>
         </is>
       </c>
-      <c r="K88" s="5" t="inlineStr"/>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+      <c r="M88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="20" customHeight="1">
       <c r="A89" s="4" t="n">
@@ -4169,7 +4351,9 @@
           <t>2026-10-18 21:43:43</t>
         </is>
       </c>
-      <c r="K89" s="5" t="inlineStr"/>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+      <c r="M89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="4" t="n">
@@ -4216,7 +4400,9 @@
           <t>2026-10-18 21:44:03</t>
         </is>
       </c>
-      <c r="K90" s="5" t="inlineStr"/>
+      <c r="K90" s="4" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr"/>
+      <c r="M90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="20" customHeight="1">
       <c r="A91" s="4" t="n">
@@ -4263,7 +4449,9 @@
           <t>2026-10-18 21:44:20</t>
         </is>
       </c>
-      <c r="K91" s="5" t="inlineStr"/>
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+      <c r="M91" s="5" t="inlineStr"/>
     </row>
     <row r="92" ht="20" customHeight="1">
       <c r="A92" s="4" t="n">
@@ -4310,7 +4498,9 @@
           <t>2026-10-18 21:44:37</t>
         </is>
       </c>
-      <c r="K92" s="5" t="inlineStr"/>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
+      <c r="M92" s="5" t="inlineStr"/>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="4" t="n">
@@ -4357,7 +4547,9 @@
           <t>2026-10-18 21:44:55</t>
         </is>
       </c>
-      <c r="K93" s="5" t="inlineStr"/>
+      <c r="K93" s="4" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+      <c r="M93" s="5" t="inlineStr"/>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="4" t="n">
@@ -4404,7 +4596,9 @@
           <t>2026-10-18 21:45:16</t>
         </is>
       </c>
-      <c r="K94" s="5" t="inlineStr"/>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+      <c r="M94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="20" customHeight="1">
       <c r="A95" s="4" t="n">
@@ -4451,7 +4645,9 @@
           <t>2026-10-18 21:45:37</t>
         </is>
       </c>
-      <c r="K95" s="5" t="inlineStr"/>
+      <c r="K95" s="4" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr"/>
+      <c r="M95" s="5" t="inlineStr"/>
     </row>
     <row r="96" ht="20" customHeight="1">
       <c r="A96" s="4" t="n">
@@ -4498,7 +4694,9 @@
           <t>2026-10-18 21:45:57</t>
         </is>
       </c>
-      <c r="K96" s="5" t="inlineStr"/>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
+      <c r="M96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="4" t="n">
@@ -4545,7 +4743,9 @@
           <t>2026-10-18 21:50:08</t>
         </is>
       </c>
-      <c r="K97" s="5" t="inlineStr">
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+      <c r="M97" s="5" t="inlineStr">
         <is>
           <t>Added on request</t>
         </is>
@@ -4553,8 +4753,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
till 10 pm 18 oct
</commit_message>
<xml_diff>
--- a/Maitry_and_Smit_Invitation_List_18_Oct.xlsx
+++ b/Maitry_and_Smit_Invitation_List_18_Oct.xlsx
@@ -558,7 +558,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Total Contacts: 94  |  Sent: 51  |  Pending: 43  |  Updated: 18-Oct-2026 10:43 PM</t>
+          <t>Total Contacts: 94  |  Sent: 61  |  Pending: 33  |  Updated: 18-Oct-2026 10:55 PM</t>
         </is>
       </c>
     </row>
@@ -2560,386 +2560,506 @@
       <c r="M45" s="12" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="8" t="n">
+      <c r="A46" s="4" t="n">
         <v>43</v>
       </c>
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>Janak.M.Surat</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D46" s="10" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>96012 91048</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
+      <c r="E46" s="6" t="inlineStr">
         <is>
           <t>99245 64844</t>
         </is>
       </c>
-      <c r="F46" s="10" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>919601291048</t>
         </is>
       </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H46" s="10" t="inlineStr"/>
-      <c r="I46" s="9" t="inlineStr"/>
-      <c r="J46" s="8" t="inlineStr"/>
-      <c r="K46" s="8" t="inlineStr"/>
-      <c r="L46" s="8" t="inlineStr"/>
-      <c r="M46" s="9" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="11" t="n">
+      <c r="A47" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B47" s="12" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Naresh.H.Dadva</t>
         </is>
       </c>
-      <c r="C47" s="11" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>97232 83070</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr"/>
-      <c r="F47" s="13" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>919723283070</t>
         </is>
       </c>
-      <c r="G47" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H47" s="13" t="inlineStr"/>
-      <c r="I47" s="12" t="inlineStr"/>
-      <c r="J47" s="11" t="inlineStr"/>
-      <c r="K47" s="11" t="inlineStr"/>
-      <c r="L47" s="11" t="inlineStr"/>
-      <c r="M47" s="12" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="8" t="n">
+      <c r="A48" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>Arvindbhai Hamabhai Mangukiya</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D48" s="10" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>84888 66704</t>
         </is>
       </c>
-      <c r="E48" s="10" t="inlineStr">
+      <c r="E48" s="6" t="inlineStr">
         <is>
           <t>99138 68477</t>
         </is>
       </c>
-      <c r="F48" s="10" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>918488866704</t>
         </is>
       </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H48" s="10" t="inlineStr"/>
-      <c r="I48" s="9" t="inlineStr"/>
-      <c r="J48" s="8" t="inlineStr"/>
-      <c r="K48" s="8" t="inlineStr"/>
-      <c r="L48" s="8" t="inlineStr"/>
-      <c r="M48" s="9" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr"/>
     </row>
     <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="11" t="n">
+      <c r="A49" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B49" s="12" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Tushar.M.Dadva.</t>
         </is>
       </c>
-      <c r="C49" s="11" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>99040 20393</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr"/>
-      <c r="F49" s="13" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>919904020393</t>
         </is>
       </c>
-      <c r="G49" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H49" s="13" t="inlineStr"/>
-      <c r="I49" s="12" t="inlineStr"/>
-      <c r="J49" s="11" t="inlineStr"/>
-      <c r="K49" s="11" t="inlineStr"/>
-      <c r="L49" s="11" t="inlineStr"/>
-      <c r="M49" s="12" t="inlineStr"/>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr"/>
+      <c r="M49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="8" t="n">
+      <c r="A50" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>Mayur M.V.Dadva</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>84600 58961</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr"/>
-      <c r="F50" s="10" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>918460058961</t>
         </is>
       </c>
-      <c r="G50" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H50" s="10" t="inlineStr"/>
-      <c r="I50" s="9" t="inlineStr"/>
-      <c r="J50" s="8" t="inlineStr"/>
-      <c r="K50" s="8" t="inlineStr"/>
-      <c r="L50" s="8" t="inlineStr"/>
-      <c r="M50" s="9" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr"/>
+      <c r="M50" s="5" t="inlineStr"/>
     </row>
     <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="11" t="n">
+      <c r="A51" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B51" s="12" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Dharmeshbhai Nathubhai</t>
         </is>
       </c>
-      <c r="C51" s="11" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D51" s="13" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>98243 48641</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr"/>
-      <c r="F51" s="13" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>919824348641</t>
         </is>
       </c>
-      <c r="G51" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H51" s="13" t="inlineStr"/>
-      <c r="I51" s="12" t="inlineStr"/>
-      <c r="J51" s="11" t="inlineStr"/>
-      <c r="K51" s="11" t="inlineStr"/>
-      <c r="L51" s="11" t="inlineStr"/>
-      <c r="M51" s="12" t="inlineStr"/>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr"/>
+      <c r="M51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="8" t="n">
+      <c r="A52" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="9" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Maheshbhai Nathubhai Mangukiya</t>
         </is>
       </c>
-      <c r="C52" s="8" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D52" s="10" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>9879881172</t>
         </is>
       </c>
-      <c r="E52" s="10" t="inlineStr"/>
-      <c r="F52" s="10" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>919879881172</t>
         </is>
       </c>
-      <c r="G52" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr"/>
-      <c r="I52" s="9" t="inlineStr"/>
-      <c r="J52" s="8" t="inlineStr"/>
-      <c r="K52" s="8" t="inlineStr"/>
-      <c r="L52" s="8" t="inlineStr"/>
-      <c r="M52" s="9" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>9825586722 (Prakashbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:53:28</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr"/>
     </row>
     <row r="53" ht="20" customHeight="1">
-      <c r="A53" s="11" t="n">
+      <c r="A53" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Dipu Janak Mangukiya</t>
         </is>
       </c>
-      <c r="C53" s="11" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D53" s="13" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>884 932 1147</t>
         </is>
       </c>
-      <c r="E53" s="13" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>88661 58204</t>
         </is>
       </c>
-      <c r="F53" s="13" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>918849321147</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H53" s="13" t="inlineStr"/>
-      <c r="I53" s="12" t="inlineStr"/>
-      <c r="J53" s="11" t="inlineStr"/>
-      <c r="K53" s="11" t="inlineStr"/>
-      <c r="L53" s="11" t="inlineStr"/>
-      <c r="M53" s="12" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>9879881172 (Maheshbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:54:24</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr"/>
+      <c r="M53" s="5" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="8" t="n">
+      <c r="A54" s="4" t="n">
         <v>51</v>
       </c>
-      <c r="B54" s="9" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Soham Naresh Mangukiya</t>
         </is>
       </c>
-      <c r="C54" s="8" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D54" s="10" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>91061 21370</t>
         </is>
       </c>
-      <c r="E54" s="10" t="inlineStr"/>
-      <c r="F54" s="10" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>919106121370</t>
         </is>
       </c>
-      <c r="G54" s="8" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H54" s="10" t="inlineStr"/>
-      <c r="I54" s="9" t="inlineStr"/>
-      <c r="J54" s="8" t="inlineStr"/>
-      <c r="K54" s="8" t="inlineStr"/>
-      <c r="L54" s="8" t="inlineStr"/>
-      <c r="M54" s="9" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>9879881172 (Maheshbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:54:47</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr"/>
+      <c r="L54" s="4" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr"/>
     </row>
     <row r="55" ht="20" customHeight="1">
-      <c r="A55" s="11" t="n">
+      <c r="A55" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Dharmik Arvind Mangukiya</t>
         </is>
       </c>
-      <c r="C55" s="11" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Sarvo</t>
         </is>
       </c>
-      <c r="D55" s="13" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>84011 44519</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr"/>
-      <c r="F55" s="13" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>918401144519</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="H55" s="13" t="inlineStr"/>
-      <c r="I55" s="12" t="inlineStr"/>
-      <c r="J55" s="11" t="inlineStr"/>
-      <c r="K55" s="11" t="inlineStr"/>
-      <c r="L55" s="11" t="inlineStr"/>
-      <c r="M55" s="12" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>9879881172 (Maheshbhai Mangukiya)</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>માંગુકિયા પરિવાર સર્વો.pdf</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-18 22:55:08</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="8" t="n">

</xml_diff>